<commit_message>
Daily recap, matchup updates, learning and research 2026-08-25
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-25.xlsx
+++ b/data/k-props/2026-08-25.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="98">
   <si>
     <t>date</t>
   </si>
@@ -157,6 +157,12 @@
     <t>Limited starter</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>Payton Tolle</t>
   </si>
   <si>
@@ -178,10 +184,16 @@
     <t>Colorado Rockies @ Washington Nationals</t>
   </si>
   <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>Will Warren</t>
   </si>
   <si>
     <t>Houston Astros @ New York Yankees</t>
+  </si>
+  <si>
+    <t>U</t>
   </si>
   <si>
     <t>Seth Lugo</t>
@@ -966,11 +978,17 @@
       <c r="Y3">
         <v>0.88</v>
       </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>-1.23</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD3">
         <v>2.27</v>
@@ -986,6 +1004,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>1.73</v>
+      </c>
+      <c r="AJ3">
+        <v>1.73</v>
+      </c>
+      <c r="AK3">
+        <v>1.73</v>
+      </c>
+      <c r="AL3">
+        <v>1.73</v>
       </c>
       <c r="AM3">
         <v>2.27</v>
@@ -996,7 +1026,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>6.5</v>
@@ -1008,13 +1038,13 @@
         <v>-137</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G4">
         <v>823826</v>
       </c>
       <c r="H4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I4">
         <v>5.6</v>
@@ -1067,8 +1097,14 @@
       <c r="Y4">
         <v>0.8824</v>
       </c>
+      <c r="Z4">
+        <v>7</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB4">
+        <v>0.12</v>
       </c>
       <c r="AC4" t="s">
         <v>44</v>
@@ -1077,7 +1113,7 @@
         <v>6.62</v>
       </c>
       <c r="AE4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AF4">
         <v>0.3041</v>
@@ -1087,6 +1123,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>0.38</v>
+      </c>
+      <c r="AJ4">
+        <v>0.38</v>
+      </c>
+      <c r="AK4">
+        <v>0.38</v>
+      </c>
+      <c r="AL4">
+        <v>0.38</v>
       </c>
       <c r="AM4">
         <v>6.62</v>
@@ -1097,7 +1145,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C5">
         <v>3.5</v>
@@ -1109,13 +1157,13 @@
         <v>116</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G5">
         <v>823826</v>
       </c>
       <c r="H5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I5">
         <v>4.5</v>
@@ -1168,8 +1216,14 @@
       <c r="Y5">
         <v>0.9777</v>
       </c>
+      <c r="Z5">
+        <v>7</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB5">
+        <v>-0.16</v>
       </c>
       <c r="AC5" t="s">
         <v>44</v>
@@ -1188,6 +1242,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>3.66</v>
+      </c>
+      <c r="AJ5">
+        <v>3.66</v>
+      </c>
+      <c r="AK5">
+        <v>3.66</v>
+      </c>
+      <c r="AL5">
+        <v>3.66</v>
       </c>
       <c r="AM5">
         <v>3.34</v>
@@ -1198,7 +1264,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1210,13 +1276,13 @@
         <v>109</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G6">
         <v>822693</v>
       </c>
       <c r="H6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I6">
         <v>4.7</v>
@@ -1269,11 +1335,17 @@
       <c r="Y6">
         <v>1.0972</v>
       </c>
+      <c r="Z6">
+        <v>6</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB6">
+        <v>1.18</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD6">
         <v>5.68</v>
@@ -1289,6 +1361,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>0.32</v>
+      </c>
+      <c r="AJ6">
+        <v>0.32</v>
+      </c>
+      <c r="AK6">
+        <v>0.32</v>
+      </c>
+      <c r="AL6">
+        <v>0.32</v>
       </c>
       <c r="AM6">
         <v>5.68</v>
@@ -1299,7 +1383,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C7">
         <v>4.5</v>
@@ -1311,13 +1395,13 @@
         <v>119</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G7">
         <v>823505</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I7">
         <v>4.9</v>
@@ -1370,8 +1454,14 @@
       <c r="Y7">
         <v>0.9612</v>
       </c>
+      <c r="Z7">
+        <v>4</v>
+      </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB7">
+        <v>0.23</v>
       </c>
       <c r="AC7" t="s">
         <v>44</v>
@@ -1390,6 +1480,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>-0.73</v>
+      </c>
+      <c r="AJ7">
+        <v>0.73</v>
+      </c>
+      <c r="AK7">
+        <v>-0.73</v>
+      </c>
+      <c r="AL7">
+        <v>0.73</v>
       </c>
       <c r="AM7">
         <v>4.73</v>
@@ -1400,7 +1502,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -1412,13 +1514,13 @@
         <v>105</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G8">
         <v>822773</v>
       </c>
       <c r="H8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I8">
         <v>5.4</v>
@@ -1471,8 +1573,14 @@
       <c r="Y8">
         <v>0.9732</v>
       </c>
+      <c r="Z8">
+        <v>5</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB8">
+        <v>0.05</v>
       </c>
       <c r="AC8" t="s">
         <v>44</v>
@@ -1491,6 +1599,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>1.45</v>
+      </c>
+      <c r="AJ8">
+        <v>1.45</v>
+      </c>
+      <c r="AK8">
+        <v>1.45</v>
+      </c>
+      <c r="AL8">
+        <v>1.45</v>
       </c>
       <c r="AM8">
         <v>3.55</v>
@@ -1501,7 +1621,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C9">
         <v>3.5</v>
@@ -1513,7 +1633,7 @@
         <v>120</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G9">
         <v>822773</v>
@@ -1572,11 +1692,17 @@
       <c r="Y9">
         <v>0.8979</v>
       </c>
+      <c r="Z9">
+        <v>4</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB9">
+        <v>-1.53</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD9">
         <v>1.97</v>
@@ -1592,6 +1718,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>2.03</v>
+      </c>
+      <c r="AJ9">
+        <v>2.03</v>
+      </c>
+      <c r="AK9">
+        <v>2.03</v>
+      </c>
+      <c r="AL9">
+        <v>2.03</v>
       </c>
       <c r="AM9">
         <v>1.97</v>
@@ -1602,7 +1740,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C10">
         <v>5.5</v>
@@ -1614,13 +1752,13 @@
         <v>120</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G10">
         <v>823585</v>
       </c>
       <c r="H10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I10">
         <v>4.8</v>
@@ -1673,11 +1811,17 @@
       <c r="Y10">
         <v>0.9313</v>
       </c>
+      <c r="Z10">
+        <v>5</v>
+      </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB10">
+        <v>-0.73</v>
       </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD10">
         <v>4.77</v>
@@ -1693,6 +1837,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>0.23</v>
+      </c>
+      <c r="AJ10">
+        <v>0.23</v>
+      </c>
+      <c r="AK10">
+        <v>0.23</v>
+      </c>
+      <c r="AL10">
+        <v>0.23</v>
       </c>
       <c r="AM10">
         <v>4.77</v>
@@ -1703,16 +1859,16 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G11">
         <v>823585</v>
       </c>
       <c r="H11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I11">
         <v>5.2</v>
@@ -1795,7 +1951,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>5.5</v>
@@ -1807,13 +1963,13 @@
         <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12">
         <v>824881</v>
       </c>
       <c r="H12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I12">
         <v>5</v>
@@ -1866,17 +2022,23 @@
       <c r="Y12">
         <v>0.9769</v>
       </c>
+      <c r="Z12">
+        <v>7</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB12">
+        <v>1.06</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD12">
         <v>6.56</v>
       </c>
       <c r="AE12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AF12">
         <v>0.3199</v>
@@ -1886,6 +2048,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>0.44</v>
+      </c>
+      <c r="AJ12">
+        <v>0.44</v>
+      </c>
+      <c r="AK12">
+        <v>0.44</v>
+      </c>
+      <c r="AL12">
+        <v>0.44</v>
       </c>
       <c r="AM12">
         <v>6.56</v>
@@ -1896,7 +2070,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -1908,13 +2082,13 @@
         <v>-152</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>824881</v>
       </c>
       <c r="H13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I13">
         <v>5.5</v>
@@ -1967,8 +2141,14 @@
       <c r="Y13">
         <v>0.9474</v>
       </c>
+      <c r="Z13">
+        <v>5</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB13">
+        <v>-0.67</v>
       </c>
       <c r="AC13" t="s">
         <v>44</v>
@@ -1987,6 +2167,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>1.17</v>
+      </c>
+      <c r="AJ13">
+        <v>1.17</v>
+      </c>
+      <c r="AK13">
+        <v>1.17</v>
+      </c>
+      <c r="AL13">
+        <v>1.17</v>
       </c>
       <c r="AM13">
         <v>3.83</v>
@@ -1997,7 +2189,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>6.5</v>
@@ -2009,13 +2201,13 @@
         <v>-105</v>
       </c>
       <c r="F14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G14">
         <v>824556</v>
       </c>
       <c r="H14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I14">
         <v>5.3</v>
@@ -2068,17 +2260,23 @@
       <c r="Y14">
         <v>1.0634</v>
       </c>
+      <c r="Z14">
+        <v>2</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB14">
+        <v>0.84</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD14">
         <v>7.94</v>
       </c>
       <c r="AE14" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AF14">
         <v>0.3048</v>
@@ -2088,6 +2286,18 @@
       </c>
       <c r="AH14">
         <v>-0.6</v>
+      </c>
+      <c r="AI14">
+        <v>-5.94</v>
+      </c>
+      <c r="AJ14">
+        <v>5.94</v>
+      </c>
+      <c r="AK14">
+        <v>-5.34</v>
+      </c>
+      <c r="AL14">
+        <v>5.34</v>
       </c>
       <c r="AM14">
         <v>7.34</v>
@@ -2098,7 +2308,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2110,13 +2320,13 @@
         <v>105</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G15">
         <v>824556</v>
       </c>
       <c r="H15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I15">
         <v>5</v>
@@ -2169,8 +2379,14 @@
       <c r="Y15">
         <v>1.046</v>
       </c>
+      <c r="Z15">
+        <v>4</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB15">
+        <v>0.68</v>
       </c>
       <c r="AC15" t="s">
         <v>44</v>
@@ -2189,6 +2405,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>-1.18</v>
+      </c>
+      <c r="AJ15">
+        <v>1.18</v>
+      </c>
+      <c r="AK15">
+        <v>-1.18</v>
+      </c>
+      <c r="AL15">
+        <v>1.18</v>
       </c>
       <c r="AM15">
         <v>5.18</v>
@@ -2199,7 +2427,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C16">
         <v>3.5</v>
@@ -2211,13 +2439,13 @@
         <v>104</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G16">
         <v>823016</v>
       </c>
       <c r="H16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I16">
         <v>4.8</v>
@@ -2270,11 +2498,17 @@
       <c r="Y16">
         <v>0.9745</v>
       </c>
+      <c r="Z16">
+        <v>5</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB16">
+        <v>-0.98</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD16">
         <v>2.52</v>
@@ -2290,6 +2524,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>2.48</v>
+      </c>
+      <c r="AJ16">
+        <v>2.48</v>
+      </c>
+      <c r="AK16">
+        <v>2.48</v>
+      </c>
+      <c r="AL16">
+        <v>2.48</v>
       </c>
       <c r="AM16">
         <v>2.52</v>
@@ -2300,16 +2546,16 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G17">
         <v>823016</v>
       </c>
       <c r="H17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I17">
         <v>5</v>
@@ -2372,7 +2618,7 @@
         <v>6.45</v>
       </c>
       <c r="AE17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AF17">
         <v>0.2507</v>
@@ -2392,7 +2638,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C18">
         <v>8.5</v>
@@ -2404,13 +2650,13 @@
         <v>-138</v>
       </c>
       <c r="F18" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G18">
         <v>823989</v>
       </c>
       <c r="H18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I18">
         <v>5.9</v>
@@ -2463,17 +2709,23 @@
       <c r="Y18">
         <v>1.0831</v>
       </c>
+      <c r="Z18">
+        <v>3</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB18">
+        <v>2.44</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD18">
         <v>11.54</v>
       </c>
       <c r="AE18" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AF18">
         <v>0.3506</v>
@@ -2483,6 +2735,18 @@
       </c>
       <c r="AH18">
         <v>-0.6</v>
+      </c>
+      <c r="AI18">
+        <v>-8.54</v>
+      </c>
+      <c r="AJ18">
+        <v>8.54</v>
+      </c>
+      <c r="AK18">
+        <v>-7.94</v>
+      </c>
+      <c r="AL18">
+        <v>7.94</v>
       </c>
       <c r="AM18">
         <v>10.94</v>
@@ -2493,7 +2757,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2505,13 +2769,13 @@
         <v>-155</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G19">
         <v>823989</v>
       </c>
       <c r="H19" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I19">
         <v>5.3</v>
@@ -2564,8 +2828,14 @@
       <c r="Y19">
         <v>0.9042</v>
       </c>
+      <c r="Z19">
+        <v>3</v>
+      </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB19">
+        <v>-0.35</v>
       </c>
       <c r="AC19" t="s">
         <v>44</v>
@@ -2584,6 +2854,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>-1.15</v>
+      </c>
+      <c r="AJ19">
+        <v>1.15</v>
+      </c>
+      <c r="AK19">
+        <v>-1.15</v>
+      </c>
+      <c r="AL19">
+        <v>1.15</v>
       </c>
       <c r="AM19">
         <v>4.15</v>
@@ -2594,7 +2876,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C20">
         <v>3.5</v>
@@ -2606,13 +2888,13 @@
         <v>-132</v>
       </c>
       <c r="F20" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G20">
         <v>825042</v>
       </c>
       <c r="H20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I20">
         <v>5.7</v>
@@ -2665,8 +2947,14 @@
       <c r="Y20">
         <v>0.88</v>
       </c>
+      <c r="Z20">
+        <v>4</v>
+      </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB20">
+        <v>-0.3</v>
       </c>
       <c r="AC20" t="s">
         <v>44</v>
@@ -2685,6 +2973,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>0.8</v>
+      </c>
+      <c r="AJ20">
+        <v>0.8</v>
+      </c>
+      <c r="AK20">
+        <v>0.8</v>
+      </c>
+      <c r="AL20">
+        <v>0.8</v>
       </c>
       <c r="AM20">
         <v>3.2</v>
@@ -2695,7 +2995,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C21">
         <v>4.5</v>
@@ -2707,13 +3007,13 @@
         <v>-135</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G21">
         <v>825042</v>
       </c>
       <c r="H21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I21">
         <v>5.9</v>
@@ -2766,8 +3066,14 @@
       <c r="Y21">
         <v>0.9663</v>
       </c>
+      <c r="Z21">
+        <v>3</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB21">
+        <v>-0.03</v>
       </c>
       <c r="AC21" t="s">
         <v>44</v>
@@ -2786,6 +3092,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-1.47</v>
+      </c>
+      <c r="AJ21">
+        <v>1.47</v>
+      </c>
+      <c r="AK21">
+        <v>-1.47</v>
+      </c>
+      <c r="AL21">
+        <v>1.47</v>
       </c>
       <c r="AM21">
         <v>4.47</v>
@@ -2796,7 +3114,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2808,13 +3126,13 @@
         <v>128</v>
       </c>
       <c r="F22" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G22">
         <v>823259</v>
       </c>
       <c r="H22" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I22">
         <v>5.3</v>
@@ -2867,8 +3185,14 @@
       <c r="Y22">
         <v>1.0063</v>
       </c>
+      <c r="Z22">
+        <v>4</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB22">
+        <v>0.12</v>
       </c>
       <c r="AC22" t="s">
         <v>44</v>
@@ -2887,6 +3211,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-1.62</v>
+      </c>
+      <c r="AJ22">
+        <v>1.62</v>
+      </c>
+      <c r="AK22">
+        <v>-1.62</v>
+      </c>
+      <c r="AL22">
+        <v>1.62</v>
       </c>
       <c r="AM22">
         <v>5.62</v>
@@ -2897,7 +3233,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>5.5</v>
@@ -2909,13 +3245,13 @@
         <v>-111</v>
       </c>
       <c r="F23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>823259</v>
       </c>
       <c r="H23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I23">
         <v>5.7</v>
@@ -2968,8 +3304,14 @@
       <c r="Y23">
         <v>1.0394</v>
       </c>
+      <c r="Z23">
+        <v>7</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB23">
+        <v>0.03</v>
       </c>
       <c r="AC23" t="s">
         <v>44</v>
@@ -2988,6 +3330,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>1.47</v>
+      </c>
+      <c r="AJ23">
+        <v>1.47</v>
+      </c>
+      <c r="AK23">
+        <v>1.47</v>
+      </c>
+      <c r="AL23">
+        <v>1.47</v>
       </c>
       <c r="AM23">
         <v>5.53</v>
@@ -2998,7 +3352,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C24">
         <v>5.5</v>
@@ -3010,13 +3364,13 @@
         <v>-104</v>
       </c>
       <c r="F24" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G24">
         <v>824962</v>
       </c>
       <c r="H24" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I24">
         <v>5.6</v>
@@ -3069,8 +3423,14 @@
       <c r="Y24">
         <v>0.9886</v>
       </c>
+      <c r="Z24">
+        <v>9</v>
+      </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB24">
+        <v>0.02</v>
       </c>
       <c r="AC24" t="s">
         <v>44</v>
@@ -3089,6 +3449,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>3.48</v>
+      </c>
+      <c r="AJ24">
+        <v>3.48</v>
+      </c>
+      <c r="AK24">
+        <v>3.48</v>
+      </c>
+      <c r="AL24">
+        <v>3.48</v>
       </c>
       <c r="AM24">
         <v>5.52</v>
@@ -3099,7 +3471,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C25">
         <v>4.5</v>
@@ -3111,13 +3483,13 @@
         <v>130</v>
       </c>
       <c r="F25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G25">
         <v>824962</v>
       </c>
       <c r="H25" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I25">
         <v>5.1</v>
@@ -3170,8 +3542,14 @@
       <c r="Y25">
         <v>0.9649</v>
       </c>
+      <c r="Z25">
+        <v>9</v>
+      </c>
       <c r="AA25" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB25">
+        <v>0.27</v>
       </c>
       <c r="AC25" t="s">
         <v>44</v>
@@ -3190,6 +3568,18 @@
       </c>
       <c r="AH25">
         <v>0</v>
+      </c>
+      <c r="AI25">
+        <v>4.23</v>
+      </c>
+      <c r="AJ25">
+        <v>4.23</v>
+      </c>
+      <c r="AK25">
+        <v>4.23</v>
+      </c>
+      <c r="AL25">
+        <v>4.23</v>
       </c>
       <c r="AM25">
         <v>4.77</v>
@@ -3200,7 +3590,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C26">
         <v>5.5</v>
@@ -3212,13 +3602,13 @@
         <v>-104</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G26">
         <v>823098</v>
       </c>
       <c r="H26" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I26">
         <v>5.3</v>
@@ -3271,17 +3661,23 @@
       <c r="Y26">
         <v>0.9915</v>
       </c>
+      <c r="Z26">
+        <v>6</v>
+      </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB26">
+        <v>1.13</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AD26">
         <v>6.63</v>
       </c>
       <c r="AE26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AF26">
         <v>0.2618</v>
@@ -3291,6 +3687,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>-0.63</v>
+      </c>
+      <c r="AJ26">
+        <v>0.63</v>
+      </c>
+      <c r="AK26">
+        <v>-0.63</v>
+      </c>
+      <c r="AL26">
+        <v>0.63</v>
       </c>
       <c r="AM26">
         <v>6.63</v>
@@ -3301,7 +3709,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C27">
         <v>4.5</v>
@@ -3313,13 +3721,13 @@
         <v>100</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G27">
         <v>823098</v>
       </c>
       <c r="H27" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I27">
         <v>5.8</v>
@@ -3372,11 +3780,17 @@
       <c r="Y27">
         <v>0.9566</v>
       </c>
+      <c r="Z27">
+        <v>7</v>
+      </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB27">
+        <v>-1.73</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD27">
         <v>2.77</v>
@@ -3392,6 +3806,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>4.23</v>
+      </c>
+      <c r="AJ27">
+        <v>4.23</v>
+      </c>
+      <c r="AK27">
+        <v>4.23</v>
+      </c>
+      <c r="AL27">
+        <v>4.23</v>
       </c>
       <c r="AM27">
         <v>2.77</v>
@@ -3402,7 +3828,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C28">
         <v>4.5</v>
@@ -3414,13 +3840,13 @@
         <v>-133</v>
       </c>
       <c r="F28" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G28">
         <v>823181</v>
       </c>
       <c r="H28" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I28">
         <v>5.3</v>
@@ -3473,8 +3899,14 @@
       <c r="Y28">
         <v>0.9304</v>
       </c>
+      <c r="Z28">
+        <v>5</v>
+      </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB28">
+        <v>-0.41</v>
       </c>
       <c r="AC28" t="s">
         <v>44</v>
@@ -3493,6 +3925,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>0.91</v>
+      </c>
+      <c r="AJ28">
+        <v>0.91</v>
+      </c>
+      <c r="AK28">
+        <v>0.91</v>
+      </c>
+      <c r="AL28">
+        <v>0.91</v>
       </c>
       <c r="AM28">
         <v>4.09</v>
@@ -3503,7 +3947,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C29">
         <v>3.5</v>
@@ -3515,13 +3959,13 @@
         <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G29">
         <v>823181</v>
       </c>
       <c r="H29" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I29">
         <v>4.8</v>
@@ -3574,11 +4018,17 @@
       <c r="Y29">
         <v>1.0996</v>
       </c>
+      <c r="Z29">
+        <v>2</v>
+      </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB29">
+        <v>1.73</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD29">
         <v>5.23</v>
@@ -3594,6 +4044,18 @@
       </c>
       <c r="AH29">
         <v>0</v>
+      </c>
+      <c r="AI29">
+        <v>-3.23</v>
+      </c>
+      <c r="AJ29">
+        <v>3.23</v>
+      </c>
+      <c r="AK29">
+        <v>-3.23</v>
+      </c>
+      <c r="AL29">
+        <v>3.23</v>
       </c>
       <c r="AM29">
         <v>5.23</v>
@@ -3604,7 +4066,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C30">
         <v>5.5</v>
@@ -3622,7 +4084,7 @@
         <v>824233</v>
       </c>
       <c r="H30" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I30">
         <v>4.7</v>
@@ -3675,8 +4137,14 @@
       <c r="Y30">
         <v>0.9633</v>
       </c>
+      <c r="Z30">
+        <v>5</v>
+      </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="AB30">
+        <v>-0.3</v>
       </c>
       <c r="AC30" t="s">
         <v>44</v>
@@ -3695,6 +4163,18 @@
       </c>
       <c r="AH30">
         <v>0</v>
+      </c>
+      <c r="AI30">
+        <v>-0.2</v>
+      </c>
+      <c r="AJ30">
+        <v>0.2</v>
+      </c>
+      <c r="AK30">
+        <v>-0.2</v>
+      </c>
+      <c r="AL30">
+        <v>0.2</v>
       </c>
       <c r="AM30">
         <v>5.2</v>
@@ -3705,7 +4185,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>4.5</v>
@@ -3717,7 +4197,7 @@
         <v>-143</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G31" t="s">
         <v>44</v>
@@ -3749,7 +4229,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>3.5</v>
@@ -3761,7 +4241,7 @@
         <v>130</v>
       </c>
       <c r="F32" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G32" t="s">
         <v>44</v>

</xml_diff>